<commit_message>
Keep rows in date order after duplicate swap; rebuild interim workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AfB9vfupsfkHsmqGpTPCDh
</commit_message>
<xml_diff>
--- a/articles_so_far.xlsx
+++ b/articles_so_far.xlsx
@@ -471,107 +471,107 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>43085</v>
+        <v>42084</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Anthony Mascarenhas</t>
+          <t>Md Shahnawaz Khan Chandan</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>GENOCIDE</t>
+          <t>Their Lips are Sealed</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/slow-reads/focus/news/genocide-1505440</t>
+          <t>https://www.thedailystar.net/in-focus/their-lips-are-sealed-72792</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>42084</v>
+        <v>42091</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Md Shahnawaz Khan Chandan</t>
+          <t>Kaberi Gayen</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Their Lips are Sealed</t>
+          <t>Why women freedom fighters are missing from Bangladesh's Liberation War films</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/their-lips-are-sealed-72792</t>
+          <t>https://www.thedailystar.net/in-focus/women-not-portrayed-freedom-fighters-screen-74241</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>42091</v>
+        <v>42098</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Kaberi Gayen</t>
+          <t>Amitava Kar</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Why women freedom fighters are missing from Bangladesh's Liberation War films</t>
+          <t>In conversation with Professor Rehman Sobhan</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/women-not-portrayed-freedom-fighters-screen-74241</t>
+          <t>https://www.thedailystar.net/in-focus/the-economist-and-the-patriot-75436</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>42098</v>
+        <v>42231</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Amitava Kar</t>
+          <t>Tarashankar Bandyopadhyay</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>In conversation with Professor Rehman Sobhan</t>
+          <t>On the Eve of the Emergence of Bangladesh</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/the-economist-and-the-patriot-75436</t>
+          <t>https://www.thedailystar.net/in-focus/the-eve-the-emergence-bangladesh-127051</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>42231</v>
+        <v>42259</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tarashankar Bandyopadhyay</t>
+          <t>The Daily Star</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>On the Eve of the Emergence of Bangladesh</t>
+          <t>A Purist's Struggle</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/the-eve-the-emergence-bangladesh-127051</t>
+          <t>https://www.thedailystar.net/in-focus/purists-struggle-141622</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>42259</v>
+        <v>42357</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -580,312 +580,312 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>A Purist's Struggle</t>
+          <t>Thinkers Will Lead The Way</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/purists-struggle-141622</t>
+          <t>https://www.thedailystar.net/slow-reads/focus/news/thinkers-will-lead-the-way-189340</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>42357</v>
+        <v>42392</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>The Daily Star</t>
+          <t>Naznin Tithi</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Thinkers Will Lead The Way</t>
+          <t>GANO ADALOT</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/slow-reads/focus/news/thinkers-will-lead-the-way-189340</t>
+          <t>https://www.thedailystar.net/in-focus/gano-adalot-205765</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>42392</v>
+        <v>42420</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Naznin Tithi</t>
+          <t>The Daily Star</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>GANO ADALOT</t>
+          <t>The Origins of the Language Movement</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/gano-adalot-205765</t>
+          <t>https://www.thedailystar.net/in-focus/the-origins-the-language-movement-574846</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>42420</v>
+        <v>42455</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>The Daily Star</t>
+          <t>Kajalie Shehreen Islam</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>The Origins of the Language Movement</t>
+          <t>The Burden of Dis/honour</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/the-origins-the-language-movement-574846</t>
+          <t>https://www.thedailystar.net/in-focus/the-burden-dishonour-1199632</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>42455</v>
+        <v>42469</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kajalie Shehreen Islam</t>
+          <t>Naeem Mohaiemen</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>The Burden of Dis/honour</t>
+          <t>Muktijuddho: Polyphony of the Ocean</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/the-burden-dishonour-1199632</t>
+          <t>https://www.thedailystar.net/in-focus/muktijuddho-polyphony-the-ocean-1206313</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>42469</v>
+        <v>42700</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Naeem Mohaiemen</t>
+          <t>ASIF MUNIER</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Muktijuddho: Polyphony of the Ocean</t>
+          <t>Munier Chowdhury: Personal Glimpses</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/muktijuddho-polyphony-the-ocean-1206313</t>
+          <t>https://www.thedailystar.net/in-focus/munier-chowdhury-personal-glimpses-1320649</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>42700</v>
+        <v>42721</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ASIF MUNIER</t>
+          <t>Serajul Islam Choudhury</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Munier Chowdhury: Personal Glimpses</t>
+          <t>THE UNFINISHED STRUGGLE</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/munier-chowdhury-personal-glimpses-1320649</t>
+          <t>https://www.thedailystar.net/in-focus/the-unfinished-struggle-1331104</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>42721</v>
+        <v>42770</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Serajul Islam Choudhury</t>
+          <t>Amitava Kar</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>THE UNFINISHED STRUGGLE</t>
+          <t>We shall overcome</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/the-unfinished-struggle-1331104</t>
+          <t>https://www.thedailystar.net/in-focus/we-shall-overcome-1355557</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>42770</v>
+        <v>42798</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amitava Kar</t>
+          <t>Md. Golam Kibria</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>We shall overcome</t>
+          <t>A Quiet Courage</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/we-shall-overcome-1355557</t>
+          <t>https://www.thedailystar.net/slow-reads/focus/news/quiet-courage-1370599</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>42798</v>
+        <v>42819</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Md. Golam Kibria</t>
+          <t>Mashruk Ahmed</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>A Quiet Courage</t>
+          <t>“The war is not over yet”</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/slow-reads/focus/news/quiet-courage-1370599</t>
+          <t>https://www.thedailystar.net/in-focus/the-war-not-over-yet-1380949</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>42819</v>
+        <v>42933</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mashruk Ahmed</t>
+          <t>Nahela Nowshin</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>“The war is not over yet”</t>
+          <t>Justice After Nuremberg</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/the-war-not-over-yet-1380949</t>
+          <t>https://www.thedailystar.net/in-focus/justice-after-nuremberg-1434352</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>42933</v>
+        <v>42961</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nahela Nowshin</t>
+          <t>Catherine Masud</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Justice After Nuremberg</t>
+          <t>Tareque and Munier: You are always with us</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/justice-after-nuremberg-1434352</t>
+          <t>https://www.thedailystar.net/in-focus/tareque-and-munier-you-are-always-us-1448296</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>42961</v>
+        <v>42996</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Catherine Masud</t>
+          <t>Sushmita S Preetha</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Tareque and Munier: You are always with us</t>
+          <t>Ethical challenges of documenting Birangonas</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/tareque-and-munier-you-are-always-us-1448296</t>
+          <t>https://www.thedailystar.net/slow-reads/focus/news/ethical-challenges-documenting-birangonas-1463638</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>42996</v>
+        <v>43045</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Sushmita S Preetha</t>
+          <t>The Daily Star</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Ethical challenges of documenting Birangonas</t>
+          <t>In loving memory of a Crack Platoon warrior</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/slow-reads/focus/news/ethical-challenges-documenting-birangonas-1463638</t>
+          <t>https://www.thedailystar.net/in-focus/loving-memory-crack-platoon-warrior-1487017</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>43045</v>
+        <v>43073</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>The Daily Star</t>
+          <t>Waqar A Khan</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>In loving memory of a Crack Platoon warrior</t>
+          <t>From the labyrinth of memory</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/loving-memory-crack-platoon-warrior-1487017</t>
+          <t>https://www.thedailystar.net/in-focus/the-labyrinth-memory-1499692</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>43073</v>
+        <v>43085</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Waqar A Khan</t>
+          <t>Anthony Mascarenhas</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>From the labyrinth of memory</t>
+          <t>GENOCIDE</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/in-focus/the-labyrinth-memory-1499692</t>
+          <t>https://www.thedailystar.net/slow-reads/focus/news/genocide-1505440</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh interim workbook after batch 14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AfB9vfupsfkHsmqGpTPCDh
</commit_message>
<xml_diff>
--- a/articles_so_far.xlsx
+++ b/articles_so_far.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Slow Reads &amp; In Focus'!$A$1:$D$165</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Other sections'!$A$1:$D$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Other sections'!$A$1:$D$291</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3927,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D137"/>
+  <dimension ref="A1:D291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5260,1426 +5260,4506 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>44242</v>
+        <v>44225</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Shah Tazrian Ashrafi</t>
+          <t>Ajoy Dasgupta</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>The Liberation War: A reading list</t>
+          <t>Opinion: 1971 to 2021 -- as Bangladesh forges ahead, Pakistan’s denial continues</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/30th-anniversary-supplements/agents-change/news/the-liberation-war-reading-list-2044793</t>
+          <t>https://www.thedailystar.net/opinion/online-exclusive/news/from-1971-to-2021-as-bangladesh-forges-ahead-pakistan-denial-continues-2036073</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>44262</v>
+        <v>44238</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>M Rafiqul Islam</t>
+          <t>Nahaly Nafisa Khan</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>The Historic Seventh March Speech of Bangabandhu: Its Influence on International Legal Discourse and Reform</t>
+          <t>How 1952 paved the way for 1971</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/law-our-rights/news/the-historic-seventh-march-speech-bangabandhu-its-influence-international-legal-discourse-and-reform-2056313</t>
+          <t>https://www.thedailystar.net/book-reviews/news/how-1952-paved-the-way-1971-2042985</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>44262</v>
+        <v>44242</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Asif Muztaba Hassan</t>
+          <t>Shah Tazrian Ashrafi</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>What makes the 7th March speech one of the best?</t>
+          <t>The Liberation War: A reading list</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/online-exclusive/news/what-makes-the-7th-march-speech-one-the-best-2056453</t>
+          <t>https://www.thedailystar.net/supplements/30th-anniversary-supplements/agents-change/news/the-liberation-war-reading-list-2044793</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>44265</v>
+        <v>44247</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Md Aminul Islam</t>
+          <t>The Daily Star</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Indomitable March: A roving treasure trove of war stories</t>
+          <t>The Spirit of 1971 – The Beginning</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/backpage/news/indomitable-march-roving-treasure-trove-war-stories-2057821</t>
+          <t>https://www.thedailystar.net/literature/news/the-spirit-1971-the-beginning-2048021</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>44278</v>
+        <v>44258</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Sanaul Huq Chowdhury</t>
+          <t>Ahmed Humayun Kabir Topu</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>The dark night memories of 25 March 1971</t>
+          <t>Mosque bears horrific memories of 1971</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/lifestyle/perspective/news/the-dark-night-memories-25-march-1971-2065057</t>
+          <t>https://www.thedailystar.net/country/news/mosque-bears-horrific-memories-1971-2054109</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>44280</v>
+        <v>44262</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Suhan Rizwan</t>
+          <t>M Rafiqul Islam</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Reflections on Muktijuddho</t>
+          <t>The Historic Seventh March Speech of Bangabandhu: Its Influence on International Legal Discourse and Reform</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/online-exclusive/reflections-bangladesh-liberation-war-1971-2066617</t>
+          <t>https://www.thedailystar.net/law-our-rights/news/the-historic-seventh-march-speech-bangabandhu-its-influence-international-legal-discourse-and-reform-2056313</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>44281</v>
+        <v>44262</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Shamsuddoza Sajen</t>
+          <t>Asif Muztaba Hassan</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Bangabandhu declares independence</t>
+          <t>What makes the 7th March speech one of the best?</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/backpage/news/bangabandhu-declares-independence-2066861</t>
+          <t>https://www.thedailystar.net/opinion/online-exclusive/news/what-makes-the-7th-march-speech-one-the-best-2056453</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>44303</v>
+        <v>44265</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Brig R P Singh, VSM (retired)</t>
+          <t>Md Aminul Islam</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>An eyewitness account of the Mujibnagar government’s swearing-in ceremony</t>
+          <t>Indomitable March: A roving treasure trove of war stories</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/news/eyewitness-account-the-mujibnagar-governments-swearing-ceremony-2078617</t>
+          <t>https://www.thedailystar.net/backpage/news/indomitable-march-roving-treasure-trove-war-stories-2057821</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>44303</v>
+        <v>44271</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Subho Basu</t>
+          <t>Shamsuddoza Sajen</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>From movement to a nation</t>
+          <t>Road to Freedom: This Day in Bangladesh Liberation War History</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/historic-mujibnagar-day/news/movement-nation-2078873</t>
+          <t>https://www.thedailystar.net/backpage/news/road-freedom-day-bangladesh-liberation-war-history-2061241</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>44303</v>
+        <v>44273</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>The Daily Star</t>
+          <t>Shamsuddoza Sajen</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>To the people of the world</t>
+          <t>Operation searchlight inked</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/historic-mujibnagar-day/news/the-people-the-world-2078881</t>
+          <t>https://www.thedailystar.net/backpage/news/operation-searchlight-inked-2062417</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>44325</v>
+        <v>44275</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Brig RP Singh, VSM (Retired)</t>
+          <t>Zakia Afrin</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Die was cast for Bangladesh’s Liberation War in April 1971</t>
+          <t>A Review of War heroines Speak: The Rape of Bangladeshi Women in 1971 War of Independence</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/news/die-was-cast-bangladeshs-liberation-war-april-1971-2090509</t>
+          <t>https://www.thedailystar.net/literature/news/review-war-heroines-speak-the-rape-bangladeshi-women-1971-war-independence-2063693</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>44364</v>
+        <v>44278</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Ishrat Jahan and Nahaly Nafisa Khan</t>
+          <t>Ali Riaz</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Remembering the Birangona: The power of personal narratives</t>
+          <t>A cancelled 1971 conference in Pakistan sends a message</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/daily-star-books/news/remembering-the-birangona-the-power-personal-narratives-2112633</t>
+          <t>https://www.thedailystar.net/opinion/black-white-grey/news/cancelled-1971-conference-pakistan-sends-message-2065033</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>44384</v>
+        <v>44278</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Brig RP Singh, VSM (Retd); Hitesh Singh</t>
+          <t>Sanaul Huq Chowdhury</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>The Kissinger-Yahya plot against Bangladesh’s liberation</t>
+          <t>The dark night memories of 25 March 1971</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/views/opinion/news/the-kissinger-yahya-plot-against-bangladeshs-liberation-2124321</t>
+          <t>https://www.thedailystar.net/lifestyle/perspective/news/the-dark-night-memories-25-march-1971-2065057</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>44406</v>
+        <v>44280</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Nahaly Nafisa Khan and Selima Sara Kabir</t>
+          <t>Partha Pratim Bhattacharjee and Wasim Bin Habib</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>The Birangona in fiction: ‘1971’ and ‘Talaash’</t>
+          <t>Operation Searchlight: Never seen so many bodies</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/books-literature/news/the-birangona-fiction-1971-and-talaash-2139686</t>
+          <t>https://www.thedailystar.net/news/bangladesh/news/operation-searchlight-never-seen-so-many-bodies-2066229</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>44546</v>
+        <v>44280</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Capt. (Retd.) Humayun Kabir Chowdhury, Bir Pratik</t>
+          <t>Suhan Rizwan</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>An ode to 1971</t>
+          <t>Reflections on Muktijuddho</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/ode-1971-2917971</t>
+          <t>https://www.thedailystar.net/online-exclusive/reflections-bangladesh-liberation-war-1971-2066617</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>44546</v>
+        <v>44281</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Mohiuddin Alamgir</t>
+          <t>Abdus Salam Shawn</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Liberated, at last</t>
+          <t>1971 in Video Games</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/liberated-last-2918636</t>
+          <t>https://www.thedailystar.net/bytes/news/1971-video-games-2067013</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>44546</v>
+        <v>44281</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Jayant Prasad</t>
+          <t>Shamsuddoza Sajen</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>The 1971 saga</t>
+          <t>Bangabandhu declares independence</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/the-1971-saga-2917976</t>
+          <t>https://www.thedailystar.net/backpage/news/bangabandhu-declares-independence-2066861</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>44637</v>
+        <v>44281</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Shams Rahman</t>
+          <t>Rasheek Tabassum Mondira</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>The Politics and Economics of Bangabandhu’s Six Points</t>
+          <t>Dhanua Kamalpur Cooperative High School: Home of sixty freedom fighters</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/views/opinion/news/the-politics-and-economics-bangabandhus-six-points-2984486</t>
+          <t>https://www.thedailystar.net/star-youth/news/dhanua-kamalpur-cooperative-high-school-home-sixty-freedom-fighters-2067181</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>44642</v>
+        <v>44281</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>M H Haider</t>
+          <t>Amanur Aman</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>The Tajuddin Ahmad persona: Tales of a Liberation War leader</t>
+          <t>Kohinoor Villa Massacre: Blood-soaked house of horror of 1971</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/life-living/news/the-tajuddin-ahmad-persona-tales-liberation-war-leader-2987246</t>
+          <t>https://www.thedailystar.net/supplements/71-memory-lane/news/kohinoor-villa-massacre-blood-soaked-house-horror-1971-2066769</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>44646</v>
+        <v>44281</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Shishir Bhattacharja</t>
+          <t>The Daily Star</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Shoronarthir Dinolipi: The diary of a 1971 refugee</t>
+          <t>Must-watch movies for a fresh perspective on the liberation war</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/celebrating-51-years-independence/news/shoronarthir-dinolipi-the-diary-1971-refugee-2990481</t>
+          <t>https://www.thedailystar.net/toggle/news/must-watch-movies-fresh-perspective-the-liberation-war-2067053</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>44654</v>
+        <v>44281</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>BSS, Dhaka</t>
+          <t>Mirza Shakil</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Kissinger who called Bangladesh 'basket case' says US role in 1971 was a 'misjudgment'</t>
+          <t>Operation Jahajmara: A turning point in the Liberation War history</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/kissinger-who-called-bangladesh-basket-case-says-us-role-1971-was-misjudgment-2997121</t>
+          <t>https://www.thedailystar.net/country/news/operation-jahajmara-turning-point-the-liberation-war-history-2067061</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>44735</v>
+        <v>44281</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Namrata</t>
+          <t>Jinat Jahan Khan</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Manash Ghosh's ' Bangladesh War': Dispatches of independence</t>
+          <t>Swadhin Bangla Betar Kendra: the source of inspiration and bravado during the liberation war</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/daily-star-books/news/dispatches-independence-3054366</t>
+          <t>https://www.thedailystar.net/tech-startup/news/swadhin-bangla-betar-kendra-the-source-inspiration-and-bravado-during-the-liberation-war-2067077</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>44909</v>
+        <v>44281</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Abdul Momin Chowdhury</t>
+          <t>Rahbar Al Haq</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>My three martyred teachers</t>
+          <t>Wheeled relics of the liberation war</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/martyred-intellectuals-day-2022/news/my-three-martyred-teachers-3195776</t>
+          <t>https://www.thedailystar.net/shift/news/wheeled-relics-the-liberation-war-2067069</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>45008</v>
+        <v>44286</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Shamsuddoza Sajen</t>
+          <t>Ashutosh Sarkar</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Reading as a form of resistance: Some anecdotes from the 1971 war</t>
+          <t>1971 War Crimes: Trials of organisations ever elusive</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/daily-star-books/news/reading-form-resistance-some-anecdotes-the-1971-war-3278586</t>
+          <t>https://www.thedailystar.net/backpage/news/1971-war-crimes-trials-organisations-ever-elusive-2069217</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>45033</v>
+        <v>44287</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Mahbub Uddin Ahmed Bir Bikram</t>
+          <t>Salil Tripathi</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Honouring Mujibnagar heroes</t>
+          <t>Modi’s Arrest in 1971: An Indian Perspective</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/focus/news/honouring-mujibnagar-heroes-3298761</t>
+          <t>https://www.thedailystar.net/opinion/news/modis-arrest-1971-indian-perspective-2069761</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>45261</v>
+        <v>44303</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Azmin Azran</t>
+          <t>The Daily Star</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Henry Kissinger’s influence on Bangladesh’s history</t>
+          <t>A Nation Rises</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/henry-kissingers-influence-bangladeshs-history-3483221</t>
+          <t>https://www.thedailystar.net/supplements/historic-mujibnagar-day/news/nation-rises-2078869</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>45276</v>
+        <v>44303</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Marina Yasmin</t>
+          <t>Brig R P Singh, VSM (retired)</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>A Testimony of Pakistan’s Cruelty, Genocide and Failure in Bangladesh</t>
+          <t>An eyewitness account of the Mujibnagar government’s swearing-in ceremony</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/victory-day-special-2023/news/testimony-pakistans-cruelty-genocide-and-failure-bangladesh-3495491</t>
+          <t>https://www.thedailystar.net/opinion/news/eyewitness-account-the-mujibnagar-governments-swearing-ceremony-2078617</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>45276</v>
+        <v>44303</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Ahmad Istiak</t>
+          <t>Subho Basu</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Battles that quickened victory</t>
+          <t>From movement to a nation</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/battles-quickened-victory-3495381</t>
+          <t>https://www.thedailystar.net/supplements/historic-mujibnagar-day/news/movement-nation-2078873</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>45277</v>
+        <v>44303</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Ahmad Istiak</t>
+          <t>Mohiuddin Alamgir</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Series genocide in 1971: Three times a survivor</t>
+          <t>Historic Mujibnagar Day: A milestone in our history</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/series-genocide-1971-three-times-survivor-3496086</t>
+          <t>https://www.thedailystar.net/frontpage/news/historic-mujibnagar-day-milestone-our-history-2078673</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>45278</v>
+        <v>44303</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>K S Nair</t>
+          <t>Tawfiq-e-Elahi Chowdhury and Bir Bikram</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Remembering 1971</t>
+          <t>Looking back: April 17, 1971</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/focus/news/remembering-1971-3497021</t>
+          <t>https://www.thedailystar.net/supplements/historic-mujibnagar-day/news/looking-back-april-17-1971-2078865</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>45358</v>
+        <v>44303</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Mahfuz Anam</t>
+          <t>Shamsuddoza Sajen</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>The speech and those transformative days of March ‘71</t>
+          <t>Mujibnagar government sworn in</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/the-third-view/news/the-speech-and-those-transformative-days-march-71-3560896</t>
+          <t>https://www.thedailystar.net/backpage/news/mujibnagar-government-sworn-2078841</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>45377</v>
+        <v>44303</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Priyam Pritim Paul</t>
+          <t>The Daily Star</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Administrative dynamics in 1971’s War of Liberation</t>
+          <t>To the people of the world</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/independence-day-special-2024/news/administrative-dynamics-1971s-war-liberation-3575151</t>
+          <t>https://www.thedailystar.net/supplements/historic-mujibnagar-day/news/the-people-the-world-2078881</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>45377</v>
+        <v>44309</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Amrin Tasnim Rafa</t>
+          <t>Shamsuddoza Sajen</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>The significance of Bangladesh's Independence Day and Victory Day</t>
+          <t>Mujibnagar cabinet meets</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/rising-stars/news/the-significance-bangladeshs-independence-day-and-victory-day-3575421</t>
+          <t>https://www.thedailystar.net/backpage/news/mujibnagar-cabinet-meets-2082201</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>45390</v>
+        <v>44325</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Khashruzzamn Choudhury</t>
+          <t>Brig RP Singh, VSM (Retired)</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>A freedom fighter’s journey to Mujibnagar</t>
+          <t>Die was cast for Bangladesh’s Liberation War in April 1971</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/focus/news/freedom-fighters-journey-mujibnagar-3584516</t>
+          <t>https://www.thedailystar.net/opinion/news/die-was-cast-bangladeshs-liberation-war-april-1971-2090509</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>45519</v>
+        <v>44360</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Ahmad Istiak</t>
+          <t>Brig RP Singh, VSM (Retd)</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Dhanmondi 32: An epicentre of independence struggle</t>
+          <t>How Mascarenhas’s report changed Bangladesh’s Liberation War</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/dhanmondi-32-epicentre-independence-struggle-3677556</t>
+          <t>https://www.thedailystar.net/opinion/news/how-mascarenhass-report-changed-bangladeshs-liberation-war-2109609</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>45641</v>
+        <v>44364</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Ahmad Istiak</t>
+          <t>Ishrat Jahan and Nahaly Nafisa Khan</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Regional Resistance: Purbo Banglar Jatiya Mukti Bahini</t>
+          <t>Remembering the Birangona: The power of personal narratives</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/regional-resistance-purbo-banglar-jatiya-mukti-bahini-3776411</t>
+          <t>https://www.thedailystar.net/daily-star-books/news/remembering-the-birangona-the-power-personal-narratives-2112633</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>45647</v>
+        <v>44384</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Anu Muhammad</t>
+          <t>Brig RP Singh, VSM (Retd); Hitesh Singh</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>The spirit of 1971: Reflections on liberation, aspirations, and modern challenges</t>
+          <t>The Kissinger-Yahya plot against Bangladesh’s liberation</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/the-spirit-1971-reflections-liberation-aspirations-and-modern-challenges-3780941</t>
+          <t>https://www.thedailystar.net/views/opinion/news/the-kissinger-yahya-plot-against-bangladeshs-liberation-2124321</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>45698</v>
+        <v>44406</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Md Abbas and Tanim Ahmed</t>
+          <t>Nahaly Nafisa Khan and Selima Sara Kabir</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Not at the cost of Muktijuddho, no way</t>
+          <t>The Birangona in fiction: ‘1971’ and ‘Talaash’</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/not-the-cost-muktijuddho-no-way-3820431</t>
+          <t>https://www.thedailystar.net/books-literature/news/the-birangona-fiction-1971-and-talaash-2139686</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>45723</v>
+        <v>44454</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Mohiuddin Alamgir</t>
+          <t>Shamsuddoza Sajen</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>‘A speech more notable for what wasn’t said’</t>
+          <t>Malraux wants to join Bangladesh Liberation War</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/speech-more-notable-what-wasnt-said-3841511</t>
+          <t>https://www.thedailystar.net/news/bangladesh/news/malraux-wants-join-bangladesh-liberation-war-2176021</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>45731</v>
+        <v>44458</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Waziha Aziz</t>
+          <t>Kamal Ahmed</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>The Birangona, un-buried</t>
+          <t>Looking back at the 1971 Concert in Sympathy</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/books-literature/news/the-birangona-un-buried-3848251</t>
+          <t>https://www.thedailystar.net/views/opinion/news/looking-back-the-1971-concert-sympathy-2178786</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>45741</v>
+        <v>44464</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Kollol Kibria</t>
+          <t>Shamsuddoza Sajen</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Henry Kissinger’s role in 1971</t>
+          <t>Mukti Bahini expanded</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/henry-kissingers-role-1971-3857056</t>
+          <t>https://www.thedailystar.net/news/bangladesh/news/mukti-bahini-expanded-2183406</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>45741</v>
+        <v>44476</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>The Daily Star</t>
+          <t>Md Shahriar Shawon</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>March 25 through the eyes of ordinary people</t>
+          <t>Reflecting on 1971 inside Prangone Mor’s ‘Condemned Cell’</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/march-25-through-the-eyes-ordinary-people-3856476</t>
+          <t>https://www.thedailystar.net/entertainment/theatre-arts/news/revisiting-1971-through-prangone-mors-condemned-cell-2192851</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>45741</v>
+        <v>44480</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Ahmad Istiak</t>
+          <t>Ashley Shoptorshi Samaddar</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Operation searchlight: The massacre at Ctg cantonment</t>
+          <t>Revisiting 9 months of the Liberation War with ‘Battle of Bangladesh’</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/operation-searchlight-the-massacre-ctg-cantonment-3856676</t>
+          <t>https://www.thedailystar.net/entertainment/theatre-arts/news/revisiting-9-months-the-liberation-war-battle-bangladesh-2195786</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>45742</v>
+        <v>44491</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Priyam Paul</t>
+          <t>Mahfuz Anam</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>1971 in Fiction: A Literary Dilemma</t>
+          <t>Column by Mahfuz Anam: Imbibing 1971 values in our post-liberation generation</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/1971-fiction-literary-dilemma-3857836</t>
+          <t>https://www.thedailystar.net/opinion/the-third-view/news/imbibing-1971-values-our-post-liberation-generation-2203316</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>45742</v>
+        <v>44494</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Shahidul Islam and Priyam Paul</t>
+          <t>Ashraf ud Doula</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Between bullets and borders Fleeing the Rajshahi massacre</t>
+          <t>A requiem for a freedom fighter</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/between-bullets-and-borders-fleeing-the-rajshahi-massacre-3857846</t>
+          <t>https://www.thedailystar.net/views/opinion/news/requiem-freedom-fighter-2205561</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>45742</v>
+        <v>44541</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Miftahul Jannat</t>
+          <t>Quazi Omar Foysal</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>Global Chords of Freedom</t>
+          <t>Bangladesh should withdraw its reservation on the UN Genocide Convention</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/global-chords-freedom-3857811</t>
+          <t>https://www.thedailystar.net/law-our-rights/news/bangladesh-should-withdraw-its-reservation-the-un-genocide-convention-2914786</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>45742</v>
+        <v>44544</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>The Daily Star</t>
+          <t>Pabitra Sarkar</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Let 1971 continue to guide our path as a nation</t>
+          <t>A Squirrel’s Tale</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/editorial/news/let-1971-continue-guide-our-path-nation-3857781</t>
+          <t>https://www.thedailystar.net/supplements/martyred-intellectuals-day-2021/news/squirrels-tale-2916751</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>45742</v>
+        <v>44544</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Lamia Karim</t>
+          <t>Subhash Mukhopadhyay</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Silencing the past</t>
+          <t>Bhai Zahir Raihan ...</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/silencing-the-past-3857856</t>
+          <t>https://www.thedailystar.net/supplements/martyred-intellectuals-day-2021/news/bhai-zahir-raihan-2916766</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>45742</v>
+        <v>44544</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Ahmad Istiak</t>
+          <t>Wasim Bin Habib</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>The legend of Nader gunda</t>
+          <t>Martyred Intellectuals Day: A loss not entirely personal</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/the-legend-nader-gunda-3857581</t>
+          <t>https://www.thedailystar.net/news/bangladesh/news/martyred-intellectuals-day-loss-not-entirely-personal-2916891</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>45742</v>
+        <v>44544</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Rahat Minhaz</t>
+          <t>Serajul Islam Choudhury</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>The People in 1971</t>
+          <t>The commitment of the martyred intellectuals</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/the-people-1971-3857821</t>
+          <t>https://www.thedailystar.net/views/opinion/news/the-commitment-the-martyred-intellectuals-2916866</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>45742</v>
+        <v>44544</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Anu Muhammad</t>
+          <t>Mahmud Shah Qureshi</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>The road to liberation: March 1971 and the years that led to it</t>
+          <t>The War of Liberation and my humble participation</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/the-road-liberation-march-1971-and-the-years-led-it-3857441</t>
+          <t>https://www.thedailystar.net/supplements/martyred-intellectuals-day-2021/news/the-war-liberation-and-my-humble-participation-2916741</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>45742</v>
+        <v>44544</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Priyam Paul</t>
+          <t>The Daily Star</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>‘The truths written in blood cannot be erased by lies’</t>
+          <t>To Opu and Topu ...</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/the-truths-written-blood-cannot-be-erased-lies-3857806</t>
+          <t>https://www.thedailystar.net/supplements/martyred-intellectuals-day-2021/news/opu-and-topu-2916771</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>45743</v>
+        <v>44546</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>The Daily Star</t>
+          <t>Muyeedul Hasan</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>Take action against fake freedom fighters</t>
+          <t>1971: PN Haksar in bridging the security gap</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/editorial/news/take-action-against-fake-freedom-fighters-3858771</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/1971-pn-haksar-bridging-the-security-gap-2917996</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>45764</v>
+        <v>44546</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Priyam Paul</t>
+          <t>Kaiser Haq</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>The Proclamation of Independence was a beacon for Bangladesh</t>
+          <t>1971: Some fragments of memory</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/the-proclamation-independence-was-beacon-bangladesh-3872661</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/1971-some-fragments-memory-2918026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>45764</v>
+        <v>44546</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Mohiuddin Alamgir</t>
+          <t>Sugata Bose</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>The spirit of Mujibnagar government can still guide us</t>
+          <t>A year of sacrificial patriotism</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/the-spirit-mujibnagar-government-can-still-guide-us-3873231</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/year-sacrificial-patriotism-2918006</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>45894</v>
+        <v>44546</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>The Daily Star</t>
+          <t>Capt. (Retd.) Humayun Kabir Chowdhury, Bir Pratik</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>No, the 1971 issues haven't been resolved</t>
+          <t>An ode to 1971</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/editorial/news/no-1971-issues-havent-been-resolved-3970561</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/ode-1971-2917971</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>45894</v>
+        <v>44546</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Mohiuddin Alamgir</t>
+          <t>Syed Jamil Ahmed, PhD</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>Why 1971 still casts a shadow in Bangladesh-Pakistan relations</t>
+          <t>How nationalist imaginaries were reconstituted in 1971</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/why-1971-still-casts-shadow-bangladesh-pakistan-relations-3970356</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/how-nationalist-imaginaries-were-reconstituted-1971-2918021</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>45949</v>
+        <v>44546</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Ayman Anika</t>
+          <t>Mohiuddin Alamgir</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>How Leesa Gazi’s work restores forgotten women’s stories from the Liberation War</t>
+          <t>Liberated, at last</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/life-living/news/how-leesa-gazis-work-restores-forgotten-womens-stories-liberation-war-4013911</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/liberated-last-2918636</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>46007</v>
+        <v>44546</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>K A S Murshid</t>
+          <t>Maisha Islam Monamee</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>The unhealed wounds of 1971: Bangladesh's unfinished liberation</t>
+          <t>Nonfiction books on the Liberation War released this year</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/unhealed-wounds-1971-bangladeshs-unfinished-liberation-4059396</t>
+          <t>https://www.thedailystar.net/daily-star-books/news/nonfiction-books-the-liberation-war-released-year-2918841</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>46049</v>
+        <v>44546</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Mohiuddin Alamgir</t>
+          <t>Dwoha Chowdhury and Mintu Deshwara</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>A witness to Bangladesh’s Liberation War</t>
+          <t>Red stains in green gardens</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/witness-bangladeshs-liberation-war-4091301</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/red-stains-green-gardens-2918616</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>46050</v>
+        <v>44546</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Rahat Minhaz</t>
+          <t>Dr. Rudabeh Shahid</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>Remembering Mark Tully, the trusted chronicler of 1971</t>
+          <t>Retracing the 1971 exodus</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/remembering-mark-tully-the-trusted-chronicler-1971-4092006</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/retracing-the-1971-exodus-2918041</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
-        <v>46053</v>
+        <v>44546</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Tahsina Nasir</t>
+          <t>Mahbub Uddin Ahmed Bir Bikram</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Oral history, 1971, and the danger of erasing memory</t>
+          <t>Tales of courage and patriotism</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/oral-history-1971-and-the-danger-erasing-memory-4094631</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/tales-courage-and-patriotism-2917981</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
-        <v>46106</v>
+        <v>44546</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Tanziral Dilshad Ditan</t>
+          <t>Jayant Prasad</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>Operation Searchlight and the unrecognised genocide of 1971</t>
+          <t>The 1971 saga</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/operation-searchlight-and-the-unrecognised-genocide-1971-4134676</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/the-1971-saga-2917976</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
-        <v>46107</v>
+        <v>44546</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Khan Khalid Adnan</t>
+          <t>Priyam Pritim Paul</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>America’s belated word on 1971, and Bangladesh’s unfinished task</t>
+          <t>The Chattogram Resistance</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/views/news/americas-belated-word-1971-and-bangladeshs-unfinished-task-4136016</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/the-chattogram-resistance-2918051</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
-        <v>46107</v>
+        <v>44546</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Azfar Hussain</t>
+          <t>Azibor Rahman</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>Independence and its discontents: For whom was 1971?</t>
+          <t>They went to sleep never to wake up</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/news/independence-and-its-discontents-whom-was-1971-4135526</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/they-went-sleep-never-wake-2918631</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
-        <v>46107</v>
+        <v>44546</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>MA Hasan</t>
+          <t>Ahmed Humayun Kabir Topu</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>The unfinished truth of 1971: Genocide, mass rape, and justice</t>
+          <t>When living is even more painful</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/news/the-unfinished-truth-1971-genocide-mass-rape-and-justice-4135531</t>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2021/news/when-living-even-more-painful-2918621</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
-        <v>46107</v>
+        <v>44546</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Khairul Hassan Jahin</t>
+          <t>Shuprova Tasneem</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>When 1971 enters the feed</t>
+          <t>‘We must stand united to uphold the spirit of our Liberation War’</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/opinion/news/when-1971-enters-the-feed-4135536</t>
+          <t>https://www.thedailystar.net/views/opinion/news/we-must-stand-united-uphold-the-spirit-our-liberation-war-2918521</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
-        <v>46107</v>
+        <v>44576</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Mohiuddin Alamgir</t>
+          <t>Tawheed Reza Noor</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Witnesses to genocide</t>
+          <t>The two-page document that recognises the 1971’s genocide</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/bangladesh/news/witnesses-genocide-4135726</t>
+          <t>https://www.thedailystar.net/law-our-rights/news/the-two-page-document-recognises-the-1971s-genocide-2939496</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
-        <v>46139</v>
+        <v>44621</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Karim Waheed</t>
+          <t>Mirza Shakil</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>Thank you, Raghu Rai, for showing me the 1971 I had not known</t>
+          <t>Tangail water tank: Mute witness to 1971 massacre</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/culture/news/thank-you-raghu-rai-showing-me-the-1971-i-had-not-known-4162106</t>
+          <t>https://www.thedailystar.net/news/bangladesh/news/tangail-water-tank-mute-witness-1971-massacre-2972621</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
-        <v>46282</v>
+        <v>44637</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Mohiuddin Alamgir</t>
+          <t>Shams Rahman</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Jamaat’s 1971 role: How the apology was repeatedly thwarted</t>
+          <t>The Politics and Economics of Bangabandhu’s Six Points</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>https://www.thedailystar.net/news/politics/news/jamaats-1971-role-how-the-apology-was-repeatedly-thwarted-4275076</t>
+          <t>https://www.thedailystar.net/views/opinion/news/the-politics-and-economics-bangabandhus-six-points-2984486</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
+        <v>44642</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>M H Haider</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>The Tajuddin Ahmad persona: Tales of a Liberation War leader</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/life-living/news/the-tajuddin-ahmad-persona-tales-liberation-war-leader-2987246</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>44646</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Priyam Paul</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>'If Pakistan acknowledges what its Army did in 1971, it will do a favour to itself'</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/celebrating-51-years-independence/news/if-pakistan-acknowledges-what-its-army-did-1971-it-will-do-favour-itself-2990476</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>44646</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Mannan Mashhur Zarif</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>London 1971 — A political frontier of the Liberation War</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/life-living/news/london-1971-political-frontier-the-liberation-war-2990981</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>44646</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Priyam Pritim Paul</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>Revisiting 1971 sagas through the lens of a silent witness</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/celebrating-51-years-independence/news/revisiting-1971-sagas-through-the-lens-silent-witness-2990456</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>44646</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Shishir Bhattacharja</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>Shoronarthir Dinolipi: The diary of a 1971 refugee</t>
+        </is>
+      </c>
+      <c r="D141" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/celebrating-51-years-independence/news/shoronarthir-dinolipi-the-diary-1971-refugee-2990481</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>44646</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Haroon Habib</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>When will UN recognise Bangladesh genocide?</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/views/opinion/news/when-will-un-recognise-bangladesh-genocide-2990536</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>44646</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Muyeedul Hasan</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>‘1971 Bangladesh – With Unbound Accounts’</t>
+        </is>
+      </c>
+      <c r="D143" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/celebrating-51-years-independence/news/1971-bangladesh-unbound-accounts-2990451</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>44654</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>BSS, Dhaka</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>Kissinger who called Bangladesh 'basket case' says US role in 1971 was a 'misjudgment'</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/kissinger-who-called-bangladesh-basket-case-says-us-role-1971-was-misjudgment-2997121</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>44666</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>EAM Asaduzzaman</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>1971 killing ground replaced by a shopping mall</t>
+        </is>
+      </c>
+      <c r="D145" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/news/1971-killing-ground-replaced-shopping-mall-3005096</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>44668</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Mohiuddin Alamgir</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>Historic Mujibnagar Day: No ordinary guard of honour</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/historic-mujibnagar-day-no-ordinary-guard-honour-3005891</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>44668</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Shams Rahman</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>Mujibnagar Day: How the Mujibnagar government turned the dream for freedom into reality</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/views/opinion/news/mujibnagar-day-how-the-mujibnagar-government-turned-the-dream-freedom-reality-3005976</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>44668</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Mahbub Uddin Ahmed Bir Bikram</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>Remembering the oath-taking of Mujibnagar government</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/online-exclusive/news/remembering-the-oath-taking-mujibnagar-government-3006526</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>44674</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Mintu Deshwara</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>History neglected: First military HQ of Liberation War at Teliapara needs proper preservation</t>
+        </is>
+      </c>
+      <c r="D149" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/news/history-neglected-first-military-hq-liberation-war-teliapara-needs-proper-preservation-3010701</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>44729</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>How much longer must the Birangonas suffer?</t>
+        </is>
+      </c>
+      <c r="D150" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/views/editorial/news/how-much-longer-must-the-birangonas-suffer-3049656</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>44735</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Namrata</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>Manash Ghosh's ' Bangladesh War': Dispatches of independence</t>
+        </is>
+      </c>
+      <c r="D151" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/daily-star-books/news/dispatches-independence-3054366</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>44833</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Zahid Akbar</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>‘Beauty Circus’: The Liberation War weaved into clever storytelling</t>
+        </is>
+      </c>
+      <c r="D152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/tv-film/news/beauty-circus-the-liberation-war-weaved-clever-storytelling-3131271</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>44854</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Kazi Zawad</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>Contradictions in a book on the Bangladesh Liberation War</t>
+        </is>
+      </c>
+      <c r="D153" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/daily-star-books/news/contradictions-book-the-bangladesh-liberation-war-3147461</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>44869</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Shuprova Tasneem</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>Guerrilla Hafiz and the freedom fighters we have failed</t>
+        </is>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/guerrilla-hafiz-and-the-freedom-fighters-we-have-failed-3160171</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>44870</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Anupam Debashis Roy</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>US resolution on 1971 genocide must get rid of divisive language</t>
+        </is>
+      </c>
+      <c r="D155" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/us-resolution-1971-genocide-must-get-rid-divisive-language-3161266</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>44883</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Sarah Anjum Bari</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>In Iffat Nawaz’s debut novel, 1971 is not an open wound</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/daily-star-books/news/iffat-nawazs-debut-novel-1971-not-open-wound-3172731</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>44909</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Kaberi Gayen</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>Legacies of Loss</t>
+        </is>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/martyred-intellectuals-day-2022/news/legacies-loss-3195766</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>44909</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>Martyred intellectuals day: Murderous scheme</t>
+        </is>
+      </c>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/martyred-intellectuals-day-murderous-scheme-3195581</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>44909</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Abdul Momin Chowdhury</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>My three martyred teachers</t>
+        </is>
+      </c>
+      <c r="D159" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/martyred-intellectuals-day-2022/news/my-three-martyred-teachers-3195776</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>44909</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Meghna Guhathakurta</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>My ’71: Experiencing Genocide, Understanding Violence</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/martyred-intellectuals-day-2022/news/my-71-experiencing-genocide-understanding-violence-3195761</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>44910</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Fabiha Afifa</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>The price of victory: 1971 and the mental health of a generation</t>
+        </is>
+      </c>
+      <c r="D161" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/shout/cover-story/news/the-price-victory-1971-and-the-mental-health-generation-3196816</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>44911</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Hrishik Roy</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>5 books to read on Victory Day</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/daily-star-books/news/5-books-read-victory-day-3197721</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>44911</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Chandrashekhar Dasgupta</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>Global diplomacy and the birth of Bangladesh</t>
+        </is>
+      </c>
+      <c r="D163" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2022/news/global-diplomacy-and-the-birth-bangladesh-3197051</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>44911</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Priyam Pritim Paul</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>Mahboobul Alam: An early historian of the 1971 war</t>
+        </is>
+      </c>
+      <c r="D164" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2022/news/mahboobul-alam-early-historian-the-1971-war-3197266</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>44911</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Mahbub Uddin Ahmed Bir Bikram</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>Mukti Bahini: The Real Heroes of Liberation War</t>
+        </is>
+      </c>
+      <c r="D165" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2022/news/mukti-bahini-the-real-heroes-liberation-war-3197061</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>44911</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Sabiba Hossain</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>Revisiting Jochna O Jononir Golpo on victory day</t>
+        </is>
+      </c>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/shout/news/revisiting-jochna-o-jononir-golpo-victory-day-3197691</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>44928</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Md Mizanur Rahman Himadri</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>'Diary of Genocide': A brief history of Martyred Intellectuals Day</t>
+        </is>
+      </c>
+      <c r="D167" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/tv-film/news/diary-genocide-brief-history-martyred-intellectuals-day-3210501</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>44934</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Tarana Halim</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>Why hasn’t the UN recognised the 1971 Bangladesh Genocide yet?</t>
+        </is>
+      </c>
+      <c r="D168" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/why-hasnt-the-un-recognised-the-1971-bangladesh-genocide-yet-3215796</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>45007</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Arun Bikash Dey</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>Chittagong College’s pivotal role in 1971</t>
+        </is>
+      </c>
+      <c r="D169" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/chattogram/news/chittagong-colleges-pivotal-role-1971-3277501</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>45008</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Shamsuddoza Sajen</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>Reading as a form of resistance: Some anecdotes from the 1971 war</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/daily-star-books/news/reading-form-resistance-some-anecdotes-the-1971-war-3278586</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>45009</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>M Rafiqul Islam</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>Factors undermining the recognition of the Bangladesh genocide</t>
+        </is>
+      </c>
+      <c r="D171" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/law-our-rights/news/factors-undermining-the-recognition-the-bangladesh-genocide-3279406</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>45010</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Ashif Ahmed Rudro</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>5 books about 25th March genocide and the aftermath</t>
+        </is>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/life-living/news/5-books-about-25th-march-genocide-and-the-aftermath-3280051</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>45010</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Tarfia Faizullah</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>Interview with a Birangona</t>
+        </is>
+      </c>
+      <c r="D173" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/star-literature/news/interview-birangona-3280216</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>45010</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Sarah Anjum Bari</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>The Birangona in poetry and conversation</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/star-literature/news/the-birangona-poetry-and-conversation-3280201</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>45010</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Shamsuddoza Sajen</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>The genocide of March 25 as a metaphor</t>
+        </is>
+      </c>
+      <c r="D175" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/the-genocide-march-25-metaphor-3279591</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>45010</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>Why won’t the UN recognise 1971 genocide?</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/editorial/news/why-wont-the-un-recognise-1971-genocide-3280396</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>45011</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Tarfia Faizullah</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>1971</t>
+        </is>
+      </c>
+      <c r="D177" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2023/news/1971-3280766</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>45011</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Nirmalendu Goon</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>A fugitive</t>
+        </is>
+      </c>
+      <c r="D178" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2023/news/fugitive-3280691</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>45011</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Shaheed Quaderi</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>Poetry, my useless weapon</t>
+        </is>
+      </c>
+      <c r="D179" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2023/news/poetry-my-useless-weapon-3280716</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>45011</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Lubaba Mahjabin Prima</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>Revisiting Iconic Movies on Bangladesh's Great Liberation War</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/tv-film/news/revisiting-iconic-movies-bangladeshs-great-liberation-war-3280951</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>45011</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Rudro Mohammad Shahidullah</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>Smell of corpse in the air</t>
+        </is>
+      </c>
+      <c r="D181" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2023/news/smell-corpse-the-air-3280711</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>45011</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Shamsur Rahman</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>You said</t>
+        </is>
+      </c>
+      <c r="D182" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2023/news/you-said-3280546</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>45011</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Kaiser Haq</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>‘FOR YOUR SAKE, O FREEDOM’ 1971 and Bangladeshi poetry</t>
+        </is>
+      </c>
+      <c r="D183" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2023/news/your-sake-o-freedom-1971-and-bangladeshi-poetry-3280541</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>45022</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Emran Mahfuz</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>War in the waters: Looking back at Operation Jackpot, 1971</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/books-literature/news/war-the-waters-looking-back-operation-jackpot-1971-3290041</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>45033</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Mahbub Uddin Ahmed Bir Bikram</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>Honouring Mujibnagar heroes</t>
+        </is>
+      </c>
+      <c r="D185" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/focus/news/honouring-mujibnagar-heroes-3298761</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>45037</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Rehman Sobhan</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>Zafrullah: Tribute to a freedom fighter and revolutionary</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/tribute/news/zafrullah-tribute-freedom-fighter-and-revolutionary-3301876</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>45044</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>The Proclamation of Independence 1971</t>
+        </is>
+      </c>
+      <c r="D187" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/law-our-rights/news/the-proclamation-independence-1971-3306236</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>45060</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Rehman Sobhan</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>Nurul Islam: Celebrating the life of a freedom fighter</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/tribute/news/nurul-islam-celebrating-the-life-freedom-fighter-3319821</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>45061</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Sara Rashid</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>Motherhood, martyrdom and the spirit of female resistance in 1971</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/daily-star-books/news/motherhood-martyrdom-and-the-spirit-female-resistance-1971-3320831</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>45099</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Zarin Tasnim</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>‘Ami Birangona Bolchi’ unveils unspoken reality</t>
+        </is>
+      </c>
+      <c r="D190" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/theatre-arts/news/ami-birangona-bolchi-unveils-unspoken-reality-3353121</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>45164</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Zahid Akbar</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>'1971 Shei Shob Din' - A riveting tale of middle-class families amidst war</t>
+        </is>
+      </c>
+      <c r="D191" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/tv-film/news/1971-shei-shob-din-riveting-tale-middle-class-families-amidst-war-3403481</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>45187</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Rafi Hossain</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>1971: Shei Shob Din: Hridi Huq’s herculean effort brings Liberation War to life</t>
+        </is>
+      </c>
+      <c r="D192" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/tv-film/news/1971-shei-shob-din-hridi-huqs-herculean-effort-brings-liberation-war-life-3421216</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>45211</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Sarazeen Saif Ahana</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>Blood, rage and love on the verge of 1971</t>
+        </is>
+      </c>
+      <c r="D193" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/daily-star-books/news/blood-rage-and-love-the-verge-1971-3441131</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>45217</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Mrinal Sircar</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>Bangladesh Genocide of 1971: Time for the West to walk the talk</t>
+        </is>
+      </c>
+      <c r="D194" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/bangladesh-genocide-1971-time-the-west-walk-the-talk-3446011</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>45261</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Azmin Azran</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>Henry Kissinger’s influence on Bangladesh’s history</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/henry-kissingers-influence-bangladeshs-history-3483221</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>45274</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>Martyred Intellectuals Day: In search of the forgotten killing fields</t>
+        </is>
+      </c>
+      <c r="D196" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/martyred-intellectuals-day-search-the-forgotten-killing-fields-3493941</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>45274</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Harry van Bommel</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>What’s holding the world back from recognising the 1971 genocide?</t>
+        </is>
+      </c>
+      <c r="D197" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/whats-holding-the-world-back-recognising-the-1971-genocide-3493931</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>45275</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>1971 War Killing Fields: Revered but not preserved</t>
+        </is>
+      </c>
+      <c r="D198" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/1971-war-killing-fields-revered-not-preserved-3494746</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>45275</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Shah Alam Shazu</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>Actor Sohel Rana recalls heroic days of Liberation War</t>
+        </is>
+      </c>
+      <c r="D199" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/tv-film/news/actor-sohel-rana-recalls-heroic-days-liberation-war-3495281</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Marina Yasmin</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>A Testimony of Pakistan’s Cruelty, Genocide and Failure in Bangladesh</t>
+        </is>
+      </c>
+      <c r="D200" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2023/news/testimony-pakistans-cruelty-genocide-and-failure-bangladesh-3495491</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>Battles that quickened victory</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/battles-quickened-victory-3495381</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Ansar Ahmed Ullah</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>Connetts risked their lives for Bangladesh in ,71</t>
+        </is>
+      </c>
+      <c r="D202" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2023/news/connetts-risked-their-lives-bangladesh-71-3495556</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>Echoes from the Archives</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2023/news/echoes-the-archives-3495576</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Momena</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>Genocide, ecology, and Zahir’s ‘Life and Political Reality’</t>
+        </is>
+      </c>
+      <c r="D204" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/star-literature/news/genocide-ecology-and-zahirs-life-and-political-reality-3495646</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Noora Shamsi Bahar</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>I, Whore; I, Birangona</t>
+        </is>
+      </c>
+      <c r="D205" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/star-literature/poetry/news/i-whore-i-birangona-3495641</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Mofidul Hoque</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>The Finale of the Bangladesh Battle</t>
+        </is>
+      </c>
+      <c r="D206" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2023/news/the-finale-the-bangladesh-battle-3495586</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Priyam Pritim Paul</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>The Heroic Role of the BMA, UK in 1971</t>
+        </is>
+      </c>
+      <c r="D207" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2023/news/the-heroic-role-the-bma-uk-1971-3495501</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Niaz Zaman</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>The Journey Home</t>
+        </is>
+      </c>
+      <c r="D208" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2023/news/the-journey-home-3495571</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>This Victory Day should be a turning point</t>
+        </is>
+      </c>
+      <c r="D209" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/editorial/news/victory-day-should-be-turning-point-3495231</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="n">
+        <v>45276</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Priyam Paul</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>“Due to a lack of firsthand experiences of the writers, there is a notable absence of works solely dedicated to our Liberation War”</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2023/news/due-lack-firsthand-experiences-the-writers-there-notable-absence-works-solely-dedicated-our-3495561</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="n">
+        <v>45277</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>Series genocide in 1971: Three times a survivor</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/series-genocide-1971-three-times-survivor-3496086</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n">
+        <v>45278</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>K S Nair</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>Remembering 1971</t>
+        </is>
+      </c>
+      <c r="D212" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/focus/news/remembering-1971-3497021</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n">
+        <v>45313</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Shah Alam Shazu</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>If I could, I would have screened ‘1971 Shei Shob Din’ in 64 districts: Hridi Huq</t>
+        </is>
+      </c>
+      <c r="D213" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/tv-film/news/if-i-could-i-would-have-screened-1971-shei-shob-din-64-districts-hridi-huq-3525406</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n">
+        <v>45330</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Ayaan Shams Siddiquee</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>Cryptic Fate back with melodic homage to 1971</t>
+        </is>
+      </c>
+      <c r="D214" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/campus/campus/news/cryptic-fate-back-melodic-homage-1971-3539341</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n">
+        <v>45330</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Fakrul Alam</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>Rehman Sobhan’s recollections of the road he took towards December 16, 1971</t>
+        </is>
+      </c>
+      <c r="D215" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/daily-star-books/news/rehman-sobhans-recollections-the-road-he-took-towards-december-16-1971-3539121</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n">
+        <v>45358</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Mahfuz Anam</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>The speech and those transformative days of March ‘71</t>
+        </is>
+      </c>
+      <c r="D216" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/the-third-view/news/the-speech-and-those-transformative-days-march-71-3560896</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>45376</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Emraan Azad</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>Challenges to the recognition of Bangladesh genocide</t>
+        </is>
+      </c>
+      <c r="D217" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/challenges-the-recognition-bangladesh-genocide-3573986</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>45377</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Ramisa Rob</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>'The Liberation War became a centre of big power rivalry'</t>
+        </is>
+      </c>
+      <c r="D218" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/geopolitical-insights/news/the-liberation-war-became-centre-big-power-rivalry-3575196</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>45377</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Priyam Pritim Paul</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>Administrative dynamics in 1971’s War of Liberation</t>
+        </is>
+      </c>
+      <c r="D219" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2024/news/administrative-dynamics-1971s-war-liberation-3575151</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>45377</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Priyam Paul and Rachel Stevens</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>Australia’s Response to the 1971 Refugee Crisis</t>
+        </is>
+      </c>
+      <c r="D220" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2024/news/australias-response-the-1971-refugee-crisis-3575126</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>45377</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Mohammad Afzalur Rahman</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>Echoes of 1971: A journey through memories</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2024/news/echoes-1971-journey-through-memories-3575181</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n">
+        <v>45377</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Muntassir Mamoon</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>Rao Farman Ali and 1971</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2024/news/rao-farman-ali-and-1971-3575166</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n">
+        <v>45377</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Amrin Tasnim Rafa</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>The significance of Bangladesh's Independence Day and Victory Day</t>
+        </is>
+      </c>
+      <c r="D223" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/rising-stars/news/the-significance-bangladeshs-independence-day-and-victory-day-3575421</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n">
+        <v>45377</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Priyam Paul</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>The untold story of Jashore’s resistance during the Liberation War</t>
+        </is>
+      </c>
+      <c r="D224" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2024/news/the-untold-story-jashores-resistance-during-the-liberation-war-3575086</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n">
+        <v>45377</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Kanak Das Gupta</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>Two Martyred Pandits: Sharada &amp; Annada Charan</t>
+        </is>
+      </c>
+      <c r="D225" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2024/news/two-martyred-pandits-sharada-annada-charan-3575171</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n">
+        <v>45390</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Khashruzzamn Choudhury</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>A freedom fighter’s journey to Mujibnagar</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/focus/news/freedom-fighters-journey-mujibnagar-3584516</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>45421</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Maliha Mashiat</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>‘Rise of Nation’: Liberation War through the ‘eyes’ of refugees at Raghu Rai’s exhibition</t>
+        </is>
+      </c>
+      <c r="D227" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/theatre-arts/news/rise-nation-liberation-war-through-the-eyes-refugees-raghu-rais-exhibition-3605911</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Dowel Biswas</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>‘I have dedicated my life to instilling the values of our Liberation war in youths’</t>
+        </is>
+      </c>
+      <c r="D228" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/theatre-arts/news/i-have-dedicated-my-life-instilling-the-values-our-liberation-war-youths-3615471</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>45480</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Tanim Ahmed</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>Freedom fighters’ quota goes against the 1971 spirit</t>
+        </is>
+      </c>
+      <c r="D229" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/freedom-fighters-quota-goes-against-the-1971-spirit-3650276</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>45519</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>Dhanmondi 32: An epicentre of independence struggle</t>
+        </is>
+      </c>
+      <c r="D230" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/dhanmondi-32-epicentre-independence-struggle-3677556</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n">
+        <v>45560</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Sadman Ahmed</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>DU student creates 1971 Liberation War time-lapse map from military perspective</t>
+        </is>
+      </c>
+      <c r="D231" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/campus/campus/news/du-student-creates-1971-liberation-war-time-lapse-map-military-perspective-3711991</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n">
+        <v>45638</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Our Correspondent, Mymensingh</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>The forgotten lens of Liberation War</t>
+        </is>
+      </c>
+      <c r="D232" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/the-forgotten-lens-liberation-war-3774166</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n">
+        <v>45640</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Kamrul Hassan Mamun</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>A Loss That Still Haunts Bangladesh</t>
+        </is>
+      </c>
+      <c r="D233" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/martyred-intellectuals-day-2024/news/loss-still-haunts-bangladesh-3775566</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n">
+        <v>45640</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Priyam Paul</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>Martyrs of Freedom</t>
+        </is>
+      </c>
+      <c r="D234" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/martyred-intellectuals-day-2024/news/martyrs-freedom-3775576</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>45640</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>Pages for freedom: Book recommendations for Victory Day</t>
+        </is>
+      </c>
+      <c r="D235" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/star-literature/news/pages-freedom-book-recommendations-victory-day-3775701</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>45640</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Nur-E-Jannat Alif</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>Poetry books to read on this Victory Day</t>
+        </is>
+      </c>
+      <c r="D236" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/life-living/news/poetry-books-read-victory-day-3776071</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n">
+        <v>45641</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>Regional Resistance: Purbo Banglar Jatiya Mukti Bahini</t>
+        </is>
+      </c>
+      <c r="D237" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/regional-resistance-purbo-banglar-jatiya-mukti-bahini-3776411</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n">
+        <v>45642</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>RBR</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>1971 War Through a Child’s Eyes: Innocence Meets Reality</t>
+        </is>
+      </c>
+      <c r="D238" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/my-dhaka/news/1971-war-through-childs-eyes-innocence-meets-reality-3777481</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n">
+        <v>45642</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Priyam Paul</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>From ‘71 to ‘24: A People United for Justice</t>
+        </is>
+      </c>
+      <c r="D239" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2024/news/71-24-people-united-justice-3777321</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n">
+        <v>45642</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Azfar Hussain</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="inlineStr">
+        <is>
+          <t>Our Victory Day and the questions of equality, justice, and human dignity</t>
+        </is>
+      </c>
+      <c r="D240" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/our-victory-day-and-the-questions-equality-justice-and-human-dignity-3776971</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n">
+        <v>45642</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Saeed Khan Shagor</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="inlineStr">
+        <is>
+          <t>Revisiting big-screen Liberation War classics</t>
+        </is>
+      </c>
+      <c r="D241" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/tv-film/news/revisiting-big-screen-liberation-war-classics-3776856</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n">
+        <v>45642</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>A.I. Mahbub Uddin Ahmed</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="inlineStr">
+        <is>
+          <t>Role of Intellectuals in Bangladesh Society, 1947-2024</t>
+        </is>
+      </c>
+      <c r="D242" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/victory-day-special-2024/news/role-intellectuals-bangladesh-society-1947-2024-3777286</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n">
+        <v>45642</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="inlineStr">
+        <is>
+          <t>Time to fulfil the dreams of 1971</t>
+        </is>
+      </c>
+      <c r="D243" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/editorial/news/time-fulfil-the-dreams-1971-3776966</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n">
+        <v>45644</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Mirza Shakil</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="inlineStr">
+        <is>
+          <t>The wonder of guerilla warfare in 1971</t>
+        </is>
+      </c>
+      <c r="D244" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/the-wonder-guerilla-warfare-1971-3778801</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n">
+        <v>45647</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Anu Muhammad</t>
+        </is>
+      </c>
+      <c r="C245" s="3" t="inlineStr">
+        <is>
+          <t>The spirit of 1971: Reflections on liberation, aspirations, and modern challenges</t>
+        </is>
+      </c>
+      <c r="D245" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/the-spirit-1971-reflections-liberation-aspirations-and-modern-challenges-3780941</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n">
+        <v>45698</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Md Abbas and Tanim Ahmed</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="inlineStr">
+        <is>
+          <t>Not at the cost of Muktijuddho, no way</t>
+        </is>
+      </c>
+      <c r="D246" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/not-the-cost-muktijuddho-no-way-3820431</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n">
+        <v>45723</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Mohiuddin Alamgir</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="inlineStr">
+        <is>
+          <t>‘A speech more notable for what wasn’t said’</t>
+        </is>
+      </c>
+      <c r="D247" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/speech-more-notable-what-wasnt-said-3841511</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n">
+        <v>45731</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Waziha Aziz</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="inlineStr">
+        <is>
+          <t>The Birangona, un-buried</t>
+        </is>
+      </c>
+      <c r="D248" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/books-literature/news/the-birangona-un-buried-3848251</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n">
+        <v>45741</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Kollol Kibria</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>Henry Kissinger’s role in 1971</t>
+        </is>
+      </c>
+      <c r="D249" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/henry-kissingers-role-1971-3857056</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n">
+        <v>45741</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="inlineStr">
+        <is>
+          <t>March 25 through the eyes of ordinary people</t>
+        </is>
+      </c>
+      <c r="D250" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/march-25-through-the-eyes-ordinary-people-3856476</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n">
+        <v>45741</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>Operation searchlight: The massacre at Ctg cantonment</t>
+        </is>
+      </c>
+      <c r="D251" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/operation-searchlight-the-massacre-ctg-cantonment-3856676</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Priyam Paul</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>1971 in Fiction: A Literary Dilemma</t>
+        </is>
+      </c>
+      <c r="D252" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/1971-fiction-literary-dilemma-3857836</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Shahidul Islam and Priyam Paul</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>Between bullets and borders Fleeing the Rajshahi massacre</t>
+        </is>
+      </c>
+      <c r="D253" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/between-bullets-and-borders-fleeing-the-rajshahi-massacre-3857846</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Miftahul Jannat</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="inlineStr">
+        <is>
+          <t>Global Chords of Freedom</t>
+        </is>
+      </c>
+      <c r="D254" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/global-chords-freedom-3857811</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>Let 1971 continue to guide our path as a nation</t>
+        </is>
+      </c>
+      <c r="D255" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/editorial/news/let-1971-continue-guide-our-path-nation-3857781</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Lamia Karim</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>Silencing the past</t>
+        </is>
+      </c>
+      <c r="D256" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/silencing-the-past-3857856</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="inlineStr">
+        <is>
+          <t>The legend of Nader gunda</t>
+        </is>
+      </c>
+      <c r="D257" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/the-legend-nader-gunda-3857581</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Rahat Minhaz</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="inlineStr">
+        <is>
+          <t>The People in 1971</t>
+        </is>
+      </c>
+      <c r="D258" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/the-people-1971-3857821</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Anu Muhammad</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>The road to liberation: March 1971 and the years that led to it</t>
+        </is>
+      </c>
+      <c r="D259" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/the-road-liberation-march-1971-and-the-years-led-it-3857441</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Priyam Paul</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>‘The truths written in blood cannot be erased by lies’</t>
+        </is>
+      </c>
+      <c r="D260" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/independence-day-special-2025/news/the-truths-written-blood-cannot-be-erased-lies-3857806</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="n">
+        <v>45743</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>Take action against fake freedom fighters</t>
+        </is>
+      </c>
+      <c r="D261" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/editorial/news/take-action-against-fake-freedom-fighters-3858771</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="n">
+        <v>45764</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Priyam Paul</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="inlineStr">
+        <is>
+          <t>The Proclamation of Independence was a beacon for Bangladesh</t>
+        </is>
+      </c>
+      <c r="D262" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/the-proclamation-independence-was-beacon-bangladesh-3872661</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="n">
+        <v>45764</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Mohiuddin Alamgir</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>The spirit of Mujibnagar government can still guide us</t>
+        </is>
+      </c>
+      <c r="D263" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/the-spirit-mujibnagar-government-can-still-guide-us-3873231</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="n">
+        <v>45894</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="inlineStr">
+        <is>
+          <t>No, the 1971 issues haven't been resolved</t>
+        </is>
+      </c>
+      <c r="D264" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/editorial/news/no-1971-issues-havent-been-resolved-3970561</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="n">
+        <v>45894</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Mohiuddin Alamgir</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>Why 1971 still casts a shadow in Bangladesh-Pakistan relations</t>
+        </is>
+      </c>
+      <c r="D265" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/why-1971-still-casts-shadow-bangladesh-pakistan-relations-3970356</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="n">
+        <v>45949</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Ayman Anika</t>
+        </is>
+      </c>
+      <c r="C266" s="3" t="inlineStr">
+        <is>
+          <t>How Leesa Gazi’s work restores forgotten women’s stories from the Liberation War</t>
+        </is>
+      </c>
+      <c r="D266" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/life-living/news/how-leesa-gazis-work-restores-forgotten-womens-stories-liberation-war-4013911</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="n">
+        <v>45997</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Our Correspondent, Benapole</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>Jashore: First district to be freed on December 6, 1971</t>
+        </is>
+      </c>
+      <c r="D267" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/jashore-first-district-be-freed-december-6-1971-4052301</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="n">
+        <v>46002</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Star Books Report</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="inlineStr">
+        <is>
+          <t>5 books that portray the ecological devastation of 1971</t>
+        </is>
+      </c>
+      <c r="D268" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/books-literature/news/5-books-portray-ecological-devastation-1971-4055736</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="n">
+        <v>46005</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Miftahul Jannat</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>A compassionate rebel in a doctor’s coat</t>
+        </is>
+      </c>
+      <c r="D269" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/supplements/martyred-intellectuals-day-2025/news/compassionate-rebel-doctors-coat-4057356</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="n">
+        <v>46005</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>The Daily Star</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="inlineStr">
+        <is>
+          <t>Martyred intellectuals are our guiding lights</t>
+        </is>
+      </c>
+      <c r="D270" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/editorial/news/martyred-intellectuals-are-our-guiding-lights-4058291</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="n">
+        <v>46005</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Mohammed Ishtiaque Khan</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>Martyred intellectuals: The torchbearers of our nation</t>
+        </is>
+      </c>
+      <c r="D271" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/martyred-intellectuals-torchbearers-our-nation-4057646</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="n">
+        <v>46005</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="inlineStr">
+        <is>
+          <t>Martyred Intellectuals’ Day: Horrors of Saidpur’s intellectual massacre</t>
+        </is>
+      </c>
+      <c r="D272" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/martyred-intellectuals-day-horrors-saidpurs-intellectual-massacre-4057741</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="n">
+        <v>46005</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Asif Bin Ali</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>What does it mean to honour the legacy of Bangladesh’s martyred intellectuals?</t>
+        </is>
+      </c>
+      <c r="D273" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/what-does-it-mean-honour-legacy-bangladeshs-martyred-intellectuals-4057641</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="n">
+        <v>46006</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C274" s="3" t="inlineStr">
+        <is>
+          <t>The funding network of 1971</t>
+        </is>
+      </c>
+      <c r="D274" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/funding-network-1971-4058551</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="n">
+        <v>46007</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Ahmad Istiak</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>From the plains to the hills: The indigenous bravery in Liberation War</t>
+        </is>
+      </c>
+      <c r="D275" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/plains-hills-indigenous-bravery-liberation-war-4059446</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="n">
+        <v>46007</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>K A S Murshid</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="inlineStr">
+        <is>
+          <t>The unhealed wounds of 1971: Bangladesh's unfinished liberation</t>
+        </is>
+      </c>
+      <c r="D276" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/unhealed-wounds-1971-bangladeshs-unfinished-liberation-4059396</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="n">
+        <v>46007</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Fahmida Khatun</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="inlineStr">
+        <is>
+          <t>Victory Day and the republic we owe ourselves</t>
+        </is>
+      </c>
+      <c r="D277" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/macro-mirror/news/victory-day-and-republic-we-owe-ourselves-4059386</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="n">
+        <v>46008</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Arts &amp; Entertainment Desk</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>When the Liberation War walked onto the stage</t>
+        </is>
+      </c>
+      <c r="D278" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/entertainment/theatre-arts/news/when-liberation-war-walked-stage-4060651</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="n">
+        <v>46017</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Iftesham Islam</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>Adieu to a frontliner of our Liberation War</t>
+        </is>
+      </c>
+      <c r="D279" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/adieu-frontliner-our-liberation-war-4066271</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="n">
+        <v>46049</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Mohiuddin Alamgir</t>
+        </is>
+      </c>
+      <c r="C280" s="3" t="inlineStr">
+        <is>
+          <t>A witness to Bangladesh’s Liberation War</t>
+        </is>
+      </c>
+      <c r="D280" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/witness-bangladeshs-liberation-war-4091301</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Rahat Minhaz</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>Remembering Mark Tully, the trusted chronicler of 1971</t>
+        </is>
+      </c>
+      <c r="D281" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/remembering-mark-tully-the-trusted-chronicler-1971-4092006</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Tahsina Nasir</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>Oral history, 1971, and the danger of erasing memory</t>
+        </is>
+      </c>
+      <c r="D282" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/oral-history-1971-and-the-danger-erasing-memory-4094631</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="n">
+        <v>46106</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Tanziral Dilshad Ditan</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>Operation Searchlight and the unrecognised genocide of 1971</t>
+        </is>
+      </c>
+      <c r="D283" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/operation-searchlight-and-the-unrecognised-genocide-1971-4134676</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Khan Khalid Adnan</t>
+        </is>
+      </c>
+      <c r="C284" s="3" t="inlineStr">
+        <is>
+          <t>America’s belated word on 1971, and Bangladesh’s unfinished task</t>
+        </is>
+      </c>
+      <c r="D284" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/views/news/americas-belated-word-1971-and-bangladeshs-unfinished-task-4136016</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Azfar Hussain</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>Independence and its discontents: For whom was 1971?</t>
+        </is>
+      </c>
+      <c r="D285" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/news/independence-and-its-discontents-whom-was-1971-4135526</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>MA Hasan</t>
+        </is>
+      </c>
+      <c r="C286" s="3" t="inlineStr">
+        <is>
+          <t>The unfinished truth of 1971: Genocide, mass rape, and justice</t>
+        </is>
+      </c>
+      <c r="D286" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/news/the-unfinished-truth-1971-genocide-mass-rape-and-justice-4135531</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Khairul Hassan Jahin</t>
+        </is>
+      </c>
+      <c r="C287" s="3" t="inlineStr">
+        <is>
+          <t>When 1971 enters the feed</t>
+        </is>
+      </c>
+      <c r="D287" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/opinion/news/when-1971-enters-the-feed-4135536</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Mohiuddin Alamgir</t>
+        </is>
+      </c>
+      <c r="C288" s="3" t="inlineStr">
+        <is>
+          <t>Witnesses to genocide</t>
+        </is>
+      </c>
+      <c r="D288" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/bangladesh/news/witnesses-genocide-4135726</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Karim Waheed</t>
+        </is>
+      </c>
+      <c r="C289" s="3" t="inlineStr">
+        <is>
+          <t>Thank you, Raghu Rai, for showing me the 1971 I had not known</t>
+        </is>
+      </c>
+      <c r="D289" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/culture/news/thank-you-raghu-rai-showing-me-the-1971-i-had-not-known-4162106</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Mohiuddin Alamgir</t>
+        </is>
+      </c>
+      <c r="C290" s="3" t="inlineStr">
+        <is>
+          <t>Jamaat’s 1971 role: How the apology was repeatedly thwarted</t>
+        </is>
+      </c>
+      <c r="D290" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thedailystar.net/news/politics/news/jamaats-1971-role-how-the-apology-was-repeatedly-thwarted-4275076</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="n">
         <v>46283</v>
       </c>
-      <c r="B137" t="inlineStr">
+      <c r="B291" t="inlineStr">
         <is>
           <t>David Bergman</t>
         </is>
       </c>
-      <c r="C137" s="3" t="inlineStr">
+      <c r="C291" s="3" t="inlineStr">
         <is>
           <t>Abdur Razzaq’s memoir: Jamaat’s internal conflict for a 1971 apology</t>
         </is>
       </c>
-      <c r="D137" s="4" t="inlineStr">
+      <c r="D291" s="4" t="inlineStr">
         <is>
           <t>https://www.thedailystar.net/opinion/views/news/abdur-razzaqs-memoir-jamaats-internal-conflict-1971-apology-4275846</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D137"/>
+  <autoFilter ref="A1:D291"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -6817,6 +9897,160 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId134"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D226" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D227" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D228" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D229" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D230" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D234" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D236" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D237" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D238" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D291" r:id="rId290"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>